<commit_message>
sync export Excel columns with Results list
</commit_message>
<xml_diff>
--- a/api/templates/export/results/en.xlsx
+++ b/api/templates/export/results/en.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="480" yWindow="480" windowWidth="20730" windowHeight="11760" tabRatio="815"/>
+    <workbookView xWindow="480" yWindow="480" windowWidth="20736" windowHeight="11760" tabRatio="815"/>
   </bookViews>
   <sheets>
     <sheet name="Results" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="55">
   <si>
     <t>Code</t>
   </si>
@@ -172,6 +172,24 @@
   </si>
   <si>
     <t>Location</t>
+  </si>
+  <si>
+    <t>Sample ID</t>
+  </si>
+  <si>
+    <t>Assay</t>
+  </si>
+  <si>
+    <t>&lt;assayName&gt;</t>
+  </si>
+  <si>
+    <t>&lt;sampleId&gt;</t>
+  </si>
+  <si>
+    <t>Result Text</t>
+  </si>
+  <si>
+    <t>&lt;resultText&gt;</t>
   </si>
 </sst>
 </file>
@@ -241,7 +259,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -264,6 +282,32 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -310,7 +354,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -352,20 +396,29 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="43">
@@ -776,23 +829,25 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F9"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:I9"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="22.5" style="5" customWidth="1"/>
-    <col min="2" max="2" width="23.125" style="7" customWidth="1"/>
-    <col min="3" max="3" width="22.375" style="8" customWidth="1"/>
+    <col min="2" max="2" width="23.09765625" style="7" customWidth="1"/>
+    <col min="3" max="3" width="22.3984375" style="8" customWidth="1"/>
     <col min="4" max="4" width="18.5" style="8" customWidth="1"/>
-    <col min="5" max="5" width="28.625" style="9" customWidth="1"/>
-    <col min="6" max="6" width="20.75" style="9" customWidth="1"/>
+    <col min="5" max="5" width="28.59765625" style="9" customWidth="1"/>
+    <col min="6" max="6" width="21.3984375" style="9" customWidth="1"/>
+    <col min="7" max="8" width="21.296875" style="9" customWidth="1"/>
+    <col min="9" max="9" width="20.69921875" style="9" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="21" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:9" ht="21" x14ac:dyDescent="0.4">
       <c r="A1" s="6" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="2" spans="1:6" s="5" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" s="5" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A2" s="5" t="s">
         <v>34</v>
       </c>
@@ -801,15 +856,21 @@
       <c r="D2" s="8"/>
       <c r="E2" s="7"/>
       <c r="F2" s="7"/>
-    </row>
-    <row r="3" spans="1:6" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="G2" s="7"/>
+      <c r="H2" s="7"/>
+      <c r="I2" s="7"/>
+    </row>
+    <row r="3" spans="1:9" s="5" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B3" s="7"/>
       <c r="C3" s="8"/>
       <c r="D3" s="8"/>
       <c r="E3" s="7"/>
       <c r="F3" s="7"/>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G3" s="7"/>
+      <c r="H3" s="7"/>
+      <c r="I3" s="7"/>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A4" s="5" t="s">
         <v>33</v>
       </c>
@@ -817,38 +878,50 @@
         <v>2</v>
       </c>
     </row>
-    <row r="5" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="15" t="s">
+    <row r="5" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="19" t="s">
         <v>40</v>
       </c>
-      <c r="B5" s="16" t="s">
+      <c r="B5" s="17" t="s">
         <v>48</v>
       </c>
-      <c r="C5" s="17"/>
-      <c r="D5" s="17"/>
-      <c r="E5" s="17"/>
-      <c r="F5" s="16" t="s">
+      <c r="C5" s="18"/>
+      <c r="D5" s="18"/>
+      <c r="E5" s="18"/>
+      <c r="F5" s="21" t="s">
+        <v>49</v>
+      </c>
+      <c r="G5" s="21" t="s">
+        <v>50</v>
+      </c>
+      <c r="H5" s="21" t="s">
+        <v>53</v>
+      </c>
+      <c r="I5" s="17" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="6" spans="1:6" s="4" customFormat="1" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="17"/>
-      <c r="B6" s="18" t="s">
+    <row r="6" spans="1:9" s="4" customFormat="1" ht="31.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="18"/>
+      <c r="B6" s="15" t="s">
         <v>37</v>
       </c>
-      <c r="C6" s="18" t="s">
+      <c r="C6" s="15" t="s">
         <v>38</v>
       </c>
-      <c r="D6" s="18" t="s">
+      <c r="D6" s="15" t="s">
         <v>42</v>
       </c>
-      <c r="E6" s="18" t="s">
+      <c r="E6" s="15" t="s">
         <v>44</v>
       </c>
-      <c r="F6" s="17"/>
-    </row>
-    <row r="7" spans="1:6" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="19" t="s">
+      <c r="F6" s="22"/>
+      <c r="G6" s="22"/>
+      <c r="H6" s="20"/>
+      <c r="I6" s="18"/>
+    </row>
+    <row r="7" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="16" t="s">
         <v>41</v>
       </c>
       <c r="B7" s="10" t="s">
@@ -863,20 +936,35 @@
       <c r="E7" s="11" t="s">
         <v>45</v>
       </c>
-      <c r="F7" s="12" t="s">
+      <c r="F7" s="11" t="s">
+        <v>52</v>
+      </c>
+      <c r="G7" s="11" t="s">
+        <v>51</v>
+      </c>
+      <c r="H7" s="11" t="s">
+        <v>54</v>
+      </c>
+      <c r="I7" s="12" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
       <c r="C9" s="13"/>
       <c r="D9" s="13"/>
       <c r="E9" s="14"/>
+      <c r="F9" s="14"/>
+      <c r="G9" s="14"/>
+      <c r="H9" s="14"/>
     </row>
   </sheetData>
-  <mergeCells count="3">
-    <mergeCell ref="F5:F6"/>
+  <mergeCells count="6">
+    <mergeCell ref="I5:I6"/>
     <mergeCell ref="B5:E5"/>
     <mergeCell ref="A5:A6"/>
+    <mergeCell ref="F5:F6"/>
+    <mergeCell ref="G5:G6"/>
+    <mergeCell ref="H5:H6"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967292" verticalDpi="4294967292" r:id="rId1"/>
@@ -891,14 +979,14 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:C27"/>
-  <sheetFormatPr defaultColWidth="8.625" defaultRowHeight="21.95" customHeight="1" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="21.9" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="5.125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="39.25" customWidth="1"/>
-    <col min="3" max="3" width="100.625" customWidth="1"/>
+    <col min="1" max="1" width="5.09765625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="39.19921875" customWidth="1"/>
+    <col min="3" max="3" width="100.59765625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -909,7 +997,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="3">
         <v>1001</v>
       </c>
@@ -920,7 +1008,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="3">
         <v>1002</v>
       </c>
@@ -931,7 +1019,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="3">
         <v>1004</v>
       </c>
@@ -942,7 +1030,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="3">
         <v>1005</v>
       </c>
@@ -953,7 +1041,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="3">
         <v>1006</v>
       </c>
@@ -964,7 +1052,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="3">
         <v>1007</v>
       </c>
@@ -975,7 +1063,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="3">
         <v>1017</v>
       </c>
@@ -986,7 +1074,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="3">
         <v>1018</v>
       </c>
@@ -997,7 +1085,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="10" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="3">
         <v>2003</v>
       </c>
@@ -1008,7 +1096,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="3">
         <v>2005</v>
       </c>
@@ -1019,7 +1107,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="12" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="3">
         <v>2008</v>
       </c>
@@ -1030,7 +1118,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="13" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="3">
         <v>2009</v>
       </c>
@@ -1041,7 +1129,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="14" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="3">
         <v>2011</v>
       </c>
@@ -1052,7 +1140,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="3">
         <v>2014</v>
       </c>
@@ -1063,7 +1151,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="16" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="3">
         <v>2016</v>
       </c>
@@ -1074,7 +1162,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="17" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="3">
         <v>2018</v>
       </c>
@@ -1085,7 +1173,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="18" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="3">
         <v>2022</v>
       </c>
@@ -1096,7 +1184,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="19" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="3">
         <v>2025</v>
       </c>
@@ -1107,7 +1195,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="20" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="3">
         <v>2032</v>
       </c>
@@ -1118,7 +1206,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="21" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="3">
         <v>2034</v>
       </c>
@@ -1129,7 +1217,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="22" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="3">
         <v>2037</v>
       </c>
@@ -1140,7 +1228,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="23" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="3">
         <v>4010</v>
       </c>
@@ -1151,7 +1239,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="24" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="3">
         <v>4017</v>
       </c>
@@ -1162,7 +1250,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="25" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="3">
         <v>5006</v>
       </c>
@@ -1173,7 +1261,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="26" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" s="3">
         <v>5007</v>
       </c>
@@ -1184,7 +1272,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="27" spans="1:3" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="3">
         <v>5011</v>
       </c>

</xml_diff>

<commit_message>
add 2 more columns in Results template
</commit_message>
<xml_diff>
--- a/api/templates/export/results/en.xlsx
+++ b/api/templates/export/results/en.xlsx
@@ -5,7 +5,7 @@
   <workbookPr showInkAnnotation="0" autoCompressPictures="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PROJECTS_2020\SystemOne\aspect\api\templates\export\results\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PROJECTS_2020\SystemOne\aspect-node-12\api\templates\export\results\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="59">
   <si>
     <t>Code</t>
   </si>
@@ -190,6 +190,18 @@
   </si>
   <si>
     <t>&lt;resultText&gt;</t>
+  </si>
+  <si>
+    <t>Workflow Status</t>
+  </si>
+  <si>
+    <t>Treatment Status</t>
+  </si>
+  <si>
+    <t>&lt;resultWorkflowStatus&gt;</t>
+  </si>
+  <si>
+    <t>&lt;resultTreatmentStatus&gt;</t>
   </si>
 </sst>
 </file>
@@ -354,7 +366,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -411,14 +423,17 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="43">
@@ -829,7 +844,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I9"/>
+  <dimension ref="A1:K9"/>
   <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="22.5" style="5" customWidth="1"/>
@@ -839,15 +854,17 @@
     <col min="5" max="5" width="28.59765625" style="9" customWidth="1"/>
     <col min="6" max="6" width="21.3984375" style="9" customWidth="1"/>
     <col min="7" max="8" width="21.296875" style="9" customWidth="1"/>
-    <col min="9" max="9" width="20.69921875" style="9" customWidth="1"/>
+    <col min="9" max="9" width="17.19921875" style="9" customWidth="1"/>
+    <col min="10" max="10" width="15.8984375" style="9" customWidth="1"/>
+    <col min="11" max="11" width="20.69921875" style="9" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="21" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:11" ht="21" x14ac:dyDescent="0.4">
       <c r="A1" s="6" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="2" spans="1:9" s="5" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:11" s="5" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A2" s="5" t="s">
         <v>34</v>
       </c>
@@ -859,8 +876,10 @@
       <c r="G2" s="7"/>
       <c r="H2" s="7"/>
       <c r="I2" s="7"/>
-    </row>
-    <row r="3" spans="1:9" s="5" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="J2" s="7"/>
+      <c r="K2" s="7"/>
+    </row>
+    <row r="3" spans="1:11" s="5" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B3" s="7"/>
       <c r="C3" s="8"/>
       <c r="D3" s="8"/>
@@ -869,8 +888,10 @@
       <c r="G3" s="7"/>
       <c r="H3" s="7"/>
       <c r="I3" s="7"/>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J3" s="7"/>
+      <c r="K3" s="7"/>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A4" s="5" t="s">
         <v>33</v>
       </c>
@@ -878,7 +899,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="5" spans="1:9" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="19" t="s">
         <v>40</v>
       </c>
@@ -888,20 +909,26 @@
       <c r="C5" s="18"/>
       <c r="D5" s="18"/>
       <c r="E5" s="18"/>
-      <c r="F5" s="21" t="s">
+      <c r="F5" s="20" t="s">
         <v>49</v>
       </c>
-      <c r="G5" s="21" t="s">
+      <c r="G5" s="20" t="s">
         <v>50</v>
       </c>
-      <c r="H5" s="21" t="s">
+      <c r="H5" s="20" t="s">
         <v>53</v>
       </c>
-      <c r="I5" s="17" t="s">
+      <c r="I5" s="20" t="s">
+        <v>55</v>
+      </c>
+      <c r="J5" s="20" t="s">
+        <v>56</v>
+      </c>
+      <c r="K5" s="17" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="6" spans="1:9" s="4" customFormat="1" ht="31.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:11" s="4" customFormat="1" ht="31.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="18"/>
       <c r="B6" s="15" t="s">
         <v>37</v>
@@ -915,12 +942,14 @@
       <c r="E6" s="15" t="s">
         <v>44</v>
       </c>
-      <c r="F6" s="22"/>
-      <c r="G6" s="22"/>
-      <c r="H6" s="20"/>
-      <c r="I6" s="18"/>
-    </row>
-    <row r="7" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="F6" s="21"/>
+      <c r="G6" s="21"/>
+      <c r="H6" s="22"/>
+      <c r="I6" s="22"/>
+      <c r="J6" s="22"/>
+      <c r="K6" s="18"/>
+    </row>
+    <row r="7" spans="1:11" s="2" customFormat="1" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="16" t="s">
         <v>41</v>
       </c>
@@ -945,26 +974,36 @@
       <c r="H7" s="11" t="s">
         <v>54</v>
       </c>
-      <c r="I7" s="12" t="s">
+      <c r="I7" s="23" t="s">
+        <v>57</v>
+      </c>
+      <c r="J7" s="23" t="s">
+        <v>58</v>
+      </c>
+      <c r="K7" s="12" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.3">
       <c r="C9" s="13"/>
       <c r="D9" s="13"/>
       <c r="E9" s="14"/>
       <c r="F9" s="14"/>
       <c r="G9" s="14"/>
       <c r="H9" s="14"/>
+      <c r="I9" s="14"/>
+      <c r="J9" s="14"/>
     </row>
   </sheetData>
-  <mergeCells count="6">
-    <mergeCell ref="I5:I6"/>
+  <mergeCells count="8">
+    <mergeCell ref="K5:K6"/>
     <mergeCell ref="B5:E5"/>
     <mergeCell ref="A5:A6"/>
     <mergeCell ref="F5:F6"/>
     <mergeCell ref="G5:G6"/>
     <mergeCell ref="H5:H6"/>
+    <mergeCell ref="I5:I6"/>
+    <mergeCell ref="J5:J6"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967292" verticalDpi="4294967292" r:id="rId1"/>

</xml_diff>

<commit_message>
add column 'Error Code'
</commit_message>
<xml_diff>
--- a/api/templates/export/results/en.xlsx
+++ b/api/templates/export/results/en.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="61">
   <si>
     <t>Code</t>
   </si>
@@ -168,9 +168,6 @@
     <t>&lt;patientId&gt;</t>
   </si>
   <si>
-    <t>Location</t>
-  </si>
-  <si>
     <t>Sample ID</t>
   </si>
   <si>
@@ -202,6 +199,15 @@
   </si>
   <si>
     <t>Sample Collection Site</t>
+  </si>
+  <si>
+    <t>Site</t>
+  </si>
+  <si>
+    <t>Error Code</t>
+  </si>
+  <si>
+    <t>&lt;errorCode&gt;</t>
   </si>
 </sst>
 </file>
@@ -844,7 +850,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:K9"/>
+  <dimension ref="A1:L9"/>
   <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="22.5" style="5" customWidth="1"/>
@@ -854,17 +860,18 @@
     <col min="5" max="5" width="28.59765625" style="9" customWidth="1"/>
     <col min="6" max="6" width="21.3984375" style="9" customWidth="1"/>
     <col min="7" max="8" width="21.296875" style="9" customWidth="1"/>
-    <col min="9" max="9" width="17.19921875" style="9" customWidth="1"/>
-    <col min="10" max="10" width="15.8984375" style="9" customWidth="1"/>
-    <col min="11" max="11" width="20.69921875" style="9" customWidth="1"/>
+    <col min="9" max="9" width="11.8984375" style="9" customWidth="1"/>
+    <col min="10" max="10" width="17.19921875" style="9" customWidth="1"/>
+    <col min="11" max="11" width="15.8984375" style="9" customWidth="1"/>
+    <col min="12" max="12" width="20.69921875" style="9" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="21" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:12" ht="21" x14ac:dyDescent="0.4">
       <c r="A1" s="6" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="2" spans="1:11" s="5" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:12" s="5" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A2" s="5" t="s">
         <v>34</v>
       </c>
@@ -878,8 +885,9 @@
       <c r="I2" s="7"/>
       <c r="J2" s="7"/>
       <c r="K2" s="7"/>
-    </row>
-    <row r="3" spans="1:11" s="5" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="L2" s="7"/>
+    </row>
+    <row r="3" spans="1:12" s="5" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B3" s="7"/>
       <c r="C3" s="8"/>
       <c r="D3" s="8"/>
@@ -890,8 +898,9 @@
       <c r="I3" s="7"/>
       <c r="J3" s="7"/>
       <c r="K3" s="7"/>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="L3" s="7"/>
+    </row>
+    <row r="4" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A4" s="5" t="s">
         <v>33</v>
       </c>
@@ -899,36 +908,39 @@
         <v>2</v>
       </c>
     </row>
-    <row r="5" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="20" t="s">
         <v>40</v>
       </c>
       <c r="B5" s="18" t="s">
-        <v>47</v>
+        <v>57</v>
       </c>
       <c r="C5" s="19"/>
       <c r="D5" s="19"/>
       <c r="E5" s="19"/>
       <c r="F5" s="21" t="s">
+        <v>47</v>
+      </c>
+      <c r="G5" s="21" t="s">
         <v>48</v>
       </c>
-      <c r="G5" s="21" t="s">
-        <v>49</v>
-      </c>
       <c r="H5" s="21" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="I5" s="21" t="s">
+        <v>59</v>
+      </c>
+      <c r="J5" s="21" t="s">
+        <v>53</v>
+      </c>
+      <c r="K5" s="21" t="s">
         <v>54</v>
       </c>
-      <c r="J5" s="21" t="s">
-        <v>55</v>
-      </c>
-      <c r="K5" s="18" t="s">
+      <c r="L5" s="18" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="6" spans="1:11" s="4" customFormat="1" ht="31.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:12" s="4" customFormat="1" ht="31.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="19"/>
       <c r="B6" s="15" t="s">
         <v>37</v>
@@ -947,9 +959,10 @@
       <c r="H6" s="23"/>
       <c r="I6" s="23"/>
       <c r="J6" s="23"/>
-      <c r="K6" s="19"/>
-    </row>
-    <row r="7" spans="1:11" s="2" customFormat="1" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="K6" s="23"/>
+      <c r="L6" s="19"/>
+    </row>
+    <row r="7" spans="1:12" s="2" customFormat="1" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="16" t="s">
         <v>41</v>
       </c>
@@ -966,25 +979,28 @@
         <v>44</v>
       </c>
       <c r="F7" s="11" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="G7" s="11" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="H7" s="11" t="s">
-        <v>53</v>
-      </c>
-      <c r="I7" s="17" t="s">
+        <v>52</v>
+      </c>
+      <c r="I7" s="11" t="s">
+        <v>60</v>
+      </c>
+      <c r="J7" s="17" t="s">
+        <v>55</v>
+      </c>
+      <c r="K7" s="17" t="s">
         <v>56</v>
       </c>
-      <c r="J7" s="17" t="s">
-        <v>57</v>
-      </c>
-      <c r="K7" s="12" t="s">
+      <c r="L7" s="12" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:12" x14ac:dyDescent="0.3">
       <c r="C9" s="13"/>
       <c r="D9" s="13"/>
       <c r="E9" s="14"/>
@@ -993,17 +1009,19 @@
       <c r="H9" s="14"/>
       <c r="I9" s="14"/>
       <c r="J9" s="14"/>
+      <c r="K9" s="14"/>
     </row>
   </sheetData>
-  <mergeCells count="8">
-    <mergeCell ref="K5:K6"/>
+  <mergeCells count="9">
+    <mergeCell ref="L5:L6"/>
     <mergeCell ref="B5:E5"/>
     <mergeCell ref="A5:A6"/>
     <mergeCell ref="F5:F6"/>
     <mergeCell ref="G5:G6"/>
     <mergeCell ref="H5:H6"/>
+    <mergeCell ref="J5:J6"/>
+    <mergeCell ref="K5:K6"/>
     <mergeCell ref="I5:I6"/>
-    <mergeCell ref="J5:J6"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967292" verticalDpi="4294967292" r:id="rId1"/>

</xml_diff>

<commit_message>
adding the flexibility of the columns to the report
</commit_message>
<xml_diff>
--- a/api/templates/export/results/en.xlsx
+++ b/api/templates/export/results/en.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="5" rupBuild="14420"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="24228"/>
   <workbookPr showInkAnnotation="0" autoCompressPictures="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PROJECTS_2020\SystemOne\aspect\api\templates\export\results\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl$\Ubuntu\home\ubuntu\aspect\api\templates\export\results\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{96FEE4F7-E4C7-43CA-9646-339CBC5929C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="480" yWindow="480" windowWidth="20736" windowHeight="11760" tabRatio="815"/>
+    <workbookView xWindow="38290" yWindow="-110" windowWidth="38620" windowHeight="21220" tabRatio="815" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Results" sheetId="1" r:id="rId1"/>
@@ -25,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="59">
   <si>
     <t>Code</t>
   </si>
@@ -178,12 +179,6 @@
   </si>
   <si>
     <t>&lt;sampleId&gt;</t>
-  </si>
-  <si>
-    <t>Result Text</t>
-  </si>
-  <si>
-    <t>&lt;resultText&gt;</t>
   </si>
   <si>
     <t>Workflow Status</t>
@@ -213,7 +208,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
   <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
@@ -443,48 +438,48 @@
     </xf>
   </cellXfs>
   <cellStyles count="43">
-    <cellStyle name="Followed Hyperlink" xfId="2" builtinId="9" hidden="1"/>
-    <cellStyle name="Followed Hyperlink" xfId="4" builtinId="9" hidden="1"/>
-    <cellStyle name="Followed Hyperlink" xfId="6" builtinId="9" hidden="1"/>
-    <cellStyle name="Followed Hyperlink" xfId="8" builtinId="9" hidden="1"/>
-    <cellStyle name="Followed Hyperlink" xfId="10" builtinId="9" hidden="1"/>
-    <cellStyle name="Followed Hyperlink" xfId="12" builtinId="9" hidden="1"/>
-    <cellStyle name="Followed Hyperlink" xfId="14" builtinId="9" hidden="1"/>
-    <cellStyle name="Followed Hyperlink" xfId="16" builtinId="9" hidden="1"/>
-    <cellStyle name="Followed Hyperlink" xfId="18" builtinId="9" hidden="1"/>
-    <cellStyle name="Followed Hyperlink" xfId="20" builtinId="9" hidden="1"/>
-    <cellStyle name="Followed Hyperlink" xfId="22" builtinId="9" hidden="1"/>
-    <cellStyle name="Followed Hyperlink" xfId="24" builtinId="9" hidden="1"/>
-    <cellStyle name="Followed Hyperlink" xfId="26" builtinId="9" hidden="1"/>
-    <cellStyle name="Followed Hyperlink" xfId="28" builtinId="9" hidden="1"/>
-    <cellStyle name="Followed Hyperlink" xfId="30" builtinId="9" hidden="1"/>
-    <cellStyle name="Followed Hyperlink" xfId="32" builtinId="9" hidden="1"/>
-    <cellStyle name="Followed Hyperlink" xfId="34" builtinId="9" hidden="1"/>
-    <cellStyle name="Followed Hyperlink" xfId="36" builtinId="9" hidden="1"/>
-    <cellStyle name="Followed Hyperlink" xfId="38" builtinId="9" hidden="1"/>
-    <cellStyle name="Followed Hyperlink" xfId="40" builtinId="9" hidden="1"/>
-    <cellStyle name="Followed Hyperlink" xfId="42" builtinId="9" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="1" builtinId="8" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="3" builtinId="8" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="5" builtinId="8" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="7" builtinId="8" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="9" builtinId="8" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="11" builtinId="8" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="13" builtinId="8" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="15" builtinId="8" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="17" builtinId="8" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="19" builtinId="8" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="21" builtinId="8" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="23" builtinId="8" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="25" builtinId="8" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="27" builtinId="8" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="29" builtinId="8" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="31" builtinId="8" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="33" builtinId="8" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="35" builtinId="8" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="37" builtinId="8" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="39" builtinId="8" hidden="1"/>
-    <cellStyle name="Hyperlink" xfId="41" builtinId="8" hidden="1"/>
+    <cellStyle name="Hipervínculo" xfId="1" builtinId="8" hidden="1"/>
+    <cellStyle name="Hipervínculo" xfId="3" builtinId="8" hidden="1"/>
+    <cellStyle name="Hipervínculo" xfId="5" builtinId="8" hidden="1"/>
+    <cellStyle name="Hipervínculo" xfId="7" builtinId="8" hidden="1"/>
+    <cellStyle name="Hipervínculo" xfId="9" builtinId="8" hidden="1"/>
+    <cellStyle name="Hipervínculo" xfId="11" builtinId="8" hidden="1"/>
+    <cellStyle name="Hipervínculo" xfId="13" builtinId="8" hidden="1"/>
+    <cellStyle name="Hipervínculo" xfId="15" builtinId="8" hidden="1"/>
+    <cellStyle name="Hipervínculo" xfId="17" builtinId="8" hidden="1"/>
+    <cellStyle name="Hipervínculo" xfId="19" builtinId="8" hidden="1"/>
+    <cellStyle name="Hipervínculo" xfId="21" builtinId="8" hidden="1"/>
+    <cellStyle name="Hipervínculo" xfId="23" builtinId="8" hidden="1"/>
+    <cellStyle name="Hipervínculo" xfId="25" builtinId="8" hidden="1"/>
+    <cellStyle name="Hipervínculo" xfId="27" builtinId="8" hidden="1"/>
+    <cellStyle name="Hipervínculo" xfId="29" builtinId="8" hidden="1"/>
+    <cellStyle name="Hipervínculo" xfId="31" builtinId="8" hidden="1"/>
+    <cellStyle name="Hipervínculo" xfId="33" builtinId="8" hidden="1"/>
+    <cellStyle name="Hipervínculo" xfId="35" builtinId="8" hidden="1"/>
+    <cellStyle name="Hipervínculo" xfId="37" builtinId="8" hidden="1"/>
+    <cellStyle name="Hipervínculo" xfId="39" builtinId="8" hidden="1"/>
+    <cellStyle name="Hipervínculo" xfId="41" builtinId="8" hidden="1"/>
+    <cellStyle name="Hipervínculo visitado" xfId="2" builtinId="9" hidden="1"/>
+    <cellStyle name="Hipervínculo visitado" xfId="4" builtinId="9" hidden="1"/>
+    <cellStyle name="Hipervínculo visitado" xfId="6" builtinId="9" hidden="1"/>
+    <cellStyle name="Hipervínculo visitado" xfId="8" builtinId="9" hidden="1"/>
+    <cellStyle name="Hipervínculo visitado" xfId="10" builtinId="9" hidden="1"/>
+    <cellStyle name="Hipervínculo visitado" xfId="12" builtinId="9" hidden="1"/>
+    <cellStyle name="Hipervínculo visitado" xfId="14" builtinId="9" hidden="1"/>
+    <cellStyle name="Hipervínculo visitado" xfId="16" builtinId="9" hidden="1"/>
+    <cellStyle name="Hipervínculo visitado" xfId="18" builtinId="9" hidden="1"/>
+    <cellStyle name="Hipervínculo visitado" xfId="20" builtinId="9" hidden="1"/>
+    <cellStyle name="Hipervínculo visitado" xfId="22" builtinId="9" hidden="1"/>
+    <cellStyle name="Hipervínculo visitado" xfId="24" builtinId="9" hidden="1"/>
+    <cellStyle name="Hipervínculo visitado" xfId="26" builtinId="9" hidden="1"/>
+    <cellStyle name="Hipervínculo visitado" xfId="28" builtinId="9" hidden="1"/>
+    <cellStyle name="Hipervínculo visitado" xfId="30" builtinId="9" hidden="1"/>
+    <cellStyle name="Hipervínculo visitado" xfId="32" builtinId="9" hidden="1"/>
+    <cellStyle name="Hipervínculo visitado" xfId="34" builtinId="9" hidden="1"/>
+    <cellStyle name="Hipervínculo visitado" xfId="36" builtinId="9" hidden="1"/>
+    <cellStyle name="Hipervínculo visitado" xfId="38" builtinId="9" hidden="1"/>
+    <cellStyle name="Hipervínculo visitado" xfId="40" builtinId="9" hidden="1"/>
+    <cellStyle name="Hipervínculo visitado" xfId="42" builtinId="9" hidden="1"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="2">
@@ -512,7 +507,7 @@
     </dxf>
   </dxfs>
   <tableStyles count="1" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4">
-    <tableStyle name="MySqlDefault" pivot="0" table="0" count="2">
+    <tableStyle name="MySqlDefault" pivot="0" table="0" count="2" xr9:uid="{00000000-0011-0000-FFFF-FFFF00000000}">
       <tableStyleElement type="wholeTable" dxfId="1"/>
       <tableStyleElement type="headerRow" dxfId="0"/>
     </tableStyle>
@@ -849,29 +844,29 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:L9"/>
-  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:K9"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="22.5" style="5" customWidth="1"/>
-    <col min="2" max="2" width="23.09765625" style="7" customWidth="1"/>
-    <col min="3" max="3" width="22.3984375" style="8" customWidth="1"/>
+    <col min="2" max="2" width="23.08203125" style="7" customWidth="1"/>
+    <col min="3" max="3" width="22.4140625" style="8" customWidth="1"/>
     <col min="4" max="4" width="18.5" style="8" customWidth="1"/>
-    <col min="5" max="5" width="28.59765625" style="9" customWidth="1"/>
-    <col min="6" max="6" width="21.3984375" style="9" customWidth="1"/>
-    <col min="7" max="8" width="21.296875" style="9" customWidth="1"/>
-    <col min="9" max="9" width="11.8984375" style="9" customWidth="1"/>
-    <col min="10" max="10" width="17.19921875" style="9" customWidth="1"/>
-    <col min="11" max="11" width="15.8984375" style="9" customWidth="1"/>
-    <col min="12" max="12" width="20.69921875" style="9" customWidth="1"/>
+    <col min="5" max="5" width="28.58203125" style="9" customWidth="1"/>
+    <col min="6" max="6" width="21.4140625" style="9" customWidth="1"/>
+    <col min="7" max="7" width="21.33203125" style="9" customWidth="1"/>
+    <col min="8" max="8" width="11.9140625" style="9" customWidth="1"/>
+    <col min="9" max="9" width="17.1640625" style="9" customWidth="1"/>
+    <col min="10" max="10" width="15.9140625" style="9" customWidth="1"/>
+    <col min="11" max="11" width="20.6640625" style="9" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="21" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:11" ht="21" x14ac:dyDescent="0.5">
       <c r="A1" s="6" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="2" spans="1:12" s="5" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:11" s="5" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A2" s="5" t="s">
         <v>34</v>
       </c>
@@ -885,9 +880,8 @@
       <c r="I2" s="7"/>
       <c r="J2" s="7"/>
       <c r="K2" s="7"/>
-      <c r="L2" s="7"/>
-    </row>
-    <row r="3" spans="1:12" s="5" customFormat="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="3" spans="1:11" s="5" customFormat="1" x14ac:dyDescent="0.35">
       <c r="B3" s="7"/>
       <c r="C3" s="8"/>
       <c r="D3" s="8"/>
@@ -898,9 +892,8 @@
       <c r="I3" s="7"/>
       <c r="J3" s="7"/>
       <c r="K3" s="7"/>
-      <c r="L3" s="7"/>
-    </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.3">
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A4" s="5" t="s">
         <v>33</v>
       </c>
@@ -908,12 +901,12 @@
         <v>2</v>
       </c>
     </row>
-    <row r="5" spans="1:12" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="20" t="s">
         <v>40</v>
       </c>
       <c r="B5" s="18" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="C5" s="19"/>
       <c r="D5" s="19"/>
@@ -925,22 +918,19 @@
         <v>48</v>
       </c>
       <c r="H5" s="21" t="s">
+        <v>57</v>
+      </c>
+      <c r="I5" s="21" t="s">
         <v>51</v>
       </c>
-      <c r="I5" s="21" t="s">
-        <v>59</v>
-      </c>
       <c r="J5" s="21" t="s">
-        <v>53</v>
-      </c>
-      <c r="K5" s="21" t="s">
-        <v>54</v>
-      </c>
-      <c r="L5" s="18" t="s">
+        <v>52</v>
+      </c>
+      <c r="K5" s="18" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="6" spans="1:12" s="4" customFormat="1" ht="31.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:11" s="4" customFormat="1" ht="31.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="19"/>
       <c r="B6" s="15" t="s">
         <v>37</v>
@@ -949,7 +939,7 @@
         <v>38</v>
       </c>
       <c r="D6" s="15" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="E6" s="15" t="s">
         <v>43</v>
@@ -959,10 +949,9 @@
       <c r="H6" s="23"/>
       <c r="I6" s="23"/>
       <c r="J6" s="23"/>
-      <c r="K6" s="23"/>
-      <c r="L6" s="19"/>
-    </row>
-    <row r="7" spans="1:12" s="2" customFormat="1" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="K6" s="19"/>
+    </row>
+    <row r="7" spans="1:11" s="2" customFormat="1" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="16" t="s">
         <v>41</v>
       </c>
@@ -985,22 +974,19 @@
         <v>49</v>
       </c>
       <c r="H7" s="11" t="s">
-        <v>52</v>
-      </c>
-      <c r="I7" s="11" t="s">
-        <v>60</v>
+        <v>58</v>
+      </c>
+      <c r="I7" s="17" t="s">
+        <v>53</v>
       </c>
       <c r="J7" s="17" t="s">
-        <v>55</v>
-      </c>
-      <c r="K7" s="17" t="s">
-        <v>56</v>
-      </c>
-      <c r="L7" s="12" t="s">
+        <v>54</v>
+      </c>
+      <c r="K7" s="12" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.35">
       <c r="C9" s="13"/>
       <c r="D9" s="13"/>
       <c r="E9" s="14"/>
@@ -1009,19 +995,17 @@
       <c r="H9" s="14"/>
       <c r="I9" s="14"/>
       <c r="J9" s="14"/>
-      <c r="K9" s="14"/>
     </row>
   </sheetData>
-  <mergeCells count="9">
-    <mergeCell ref="L5:L6"/>
+  <mergeCells count="8">
+    <mergeCell ref="K5:K6"/>
     <mergeCell ref="B5:E5"/>
     <mergeCell ref="A5:A6"/>
     <mergeCell ref="F5:F6"/>
     <mergeCell ref="G5:G6"/>
+    <mergeCell ref="I5:I6"/>
+    <mergeCell ref="J5:J6"/>
     <mergeCell ref="H5:H6"/>
-    <mergeCell ref="J5:J6"/>
-    <mergeCell ref="K5:K6"/>
-    <mergeCell ref="I5:I6"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967292" verticalDpi="4294967292" r:id="rId1"/>
@@ -1034,16 +1018,16 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:C27"/>
-  <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="21.9" customHeight="1" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.58203125" defaultRowHeight="21.9" customHeight="1" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="5.09765625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="39.19921875" customWidth="1"/>
-    <col min="3" max="3" width="100.59765625" customWidth="1"/>
+    <col min="1" max="1" width="5.08203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="39.1640625" customWidth="1"/>
+    <col min="3" max="3" width="100.58203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1054,7 +1038,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="3">
         <v>1001</v>
       </c>
@@ -1065,7 +1049,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A3" s="3">
         <v>1002</v>
       </c>
@@ -1076,7 +1060,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="3">
         <v>1004</v>
       </c>
@@ -1087,7 +1071,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A5" s="3">
         <v>1005</v>
       </c>
@@ -1098,7 +1082,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A6" s="3">
         <v>1006</v>
       </c>
@@ -1109,7 +1093,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A7" s="3">
         <v>1007</v>
       </c>
@@ -1120,7 +1104,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A8" s="3">
         <v>1017</v>
       </c>
@@ -1131,7 +1115,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="3">
         <v>1018</v>
       </c>
@@ -1142,7 +1126,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="10" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="3">
         <v>2003</v>
       </c>
@@ -1153,7 +1137,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="3">
         <v>2005</v>
       </c>
@@ -1164,7 +1148,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="12" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="3">
         <v>2008</v>
       </c>
@@ -1175,7 +1159,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="13" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="3">
         <v>2009</v>
       </c>
@@ -1186,7 +1170,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="14" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A14" s="3">
         <v>2011</v>
       </c>
@@ -1197,7 +1181,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A15" s="3">
         <v>2014</v>
       </c>
@@ -1208,7 +1192,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="16" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A16" s="3">
         <v>2016</v>
       </c>
@@ -1219,7 +1203,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="17" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A17" s="3">
         <v>2018</v>
       </c>
@@ -1230,7 +1214,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="18" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A18" s="3">
         <v>2022</v>
       </c>
@@ -1241,7 +1225,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="19" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A19" s="3">
         <v>2025</v>
       </c>
@@ -1252,7 +1236,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="20" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A20" s="3">
         <v>2032</v>
       </c>
@@ -1263,7 +1247,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="21" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A21" s="3">
         <v>2034</v>
       </c>
@@ -1274,7 +1258,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="22" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A22" s="3">
         <v>2037</v>
       </c>
@@ -1285,7 +1269,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="23" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A23" s="3">
         <v>4010</v>
       </c>
@@ -1296,7 +1280,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="24" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A24" s="3">
         <v>4017</v>
       </c>
@@ -1307,7 +1291,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="25" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A25" s="3">
         <v>5006</v>
       </c>
@@ -1318,7 +1302,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="26" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A26" s="3">
         <v>5007</v>
       </c>
@@ -1329,7 +1313,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="27" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:3" ht="21.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A27" s="3">
         <v>5011</v>
       </c>

</xml_diff>

<commit_message>
Change the template for export
</commit_message>
<xml_diff>
--- a/api/templates/export/results/en.xlsx
+++ b/api/templates/export/results/en.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="24228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="24701"/>
   <workbookPr showInkAnnotation="0" autoCompressPictures="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl$\Ubuntu\home\ubuntu\aspect\api\templates\export\results\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-20.04\home\ubuntu\aspect\api\templates\all_results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{96FEE4F7-E4C7-43CA-9646-339CBC5929C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{70F6B89A-9786-4A8E-A7AA-8CCDC0C77FF0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38290" yWindow="-110" windowWidth="38620" windowHeight="21220" tabRatio="815" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="5340" yWindow="5340" windowWidth="28800" windowHeight="15410" tabRatio="815" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Results" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="60">
   <si>
     <t>Code</t>
   </si>
@@ -130,9 +130,6 @@
     <t>&lt;Table&gt;</t>
   </si>
   <si>
-    <t>Printed on &lt;date&gt;</t>
-  </si>
-  <si>
     <t>Aspect Results</t>
   </si>
   <si>
@@ -203,13 +200,19 @@
   </si>
   <si>
     <t>&lt;errorCode&gt;</t>
+  </si>
+  <si>
+    <t>Printed on &lt;Dates&gt;</t>
+  </si>
+  <si>
+    <t>There are &lt;PerformanceTotalRecordLimit&gt; more records, but report size is limited to &lt;PerformanceQueryLimit&gt; records for performance reasons. If you need more results please filter them by any of the possible filters we are providing.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -257,8 +260,15 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C0006"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -269,6 +279,11 @@
       <patternFill patternType="solid">
         <fgColor theme="6" tint="0.59999389629810485"/>
         <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
       </patternFill>
     </fill>
   </fills>
@@ -322,7 +337,7 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="43">
+  <cellStyleXfs count="44">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
@@ -366,8 +381,9 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -436,8 +452,11 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="43" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="43">
+  <cellStyles count="44">
     <cellStyle name="Hipervínculo" xfId="1" builtinId="8" hidden="1"/>
     <cellStyle name="Hipervínculo" xfId="3" builtinId="8" hidden="1"/>
     <cellStyle name="Hipervínculo" xfId="5" builtinId="8" hidden="1"/>
@@ -480,6 +499,7 @@
     <cellStyle name="Hipervínculo visitado" xfId="38" builtinId="9" hidden="1"/>
     <cellStyle name="Hipervínculo visitado" xfId="40" builtinId="9" hidden="1"/>
     <cellStyle name="Hipervínculo visitado" xfId="42" builtinId="9" hidden="1"/>
+    <cellStyle name="Incorrecto" xfId="43" builtinId="27"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="2">
@@ -845,7 +865,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K9"/>
+  <dimension ref="A1:K10"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="22.5" style="5" customWidth="1"/>
@@ -863,12 +883,12 @@
   <sheetData>
     <row r="1" spans="1:11" ht="21" x14ac:dyDescent="0.5">
       <c r="A1" s="6" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="2" spans="1:11" s="5" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A2" s="5" t="s">
-        <v>34</v>
+        <v>58</v>
       </c>
       <c r="B2" s="7"/>
       <c r="C2" s="8"/>
@@ -881,131 +901,147 @@
       <c r="J2" s="7"/>
       <c r="K2" s="7"/>
     </row>
-    <row r="3" spans="1:11" s="5" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="B3" s="7"/>
-      <c r="C3" s="8"/>
-      <c r="D3" s="8"/>
-      <c r="E3" s="7"/>
-      <c r="F3" s="7"/>
-      <c r="G3" s="7"/>
-      <c r="H3" s="7"/>
-      <c r="I3" s="7"/>
-      <c r="J3" s="7"/>
-      <c r="K3" s="7"/>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A4" s="5" t="s">
+    <row r="3" spans="1:11" s="5" customFormat="1" ht="29" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A3" s="24" t="s">
+        <v>59</v>
+      </c>
+      <c r="B3" s="24"/>
+      <c r="C3" s="24"/>
+      <c r="D3" s="24"/>
+      <c r="E3" s="24"/>
+      <c r="F3" s="24"/>
+      <c r="G3" s="24"/>
+      <c r="H3" s="24"/>
+      <c r="I3" s="24"/>
+      <c r="J3" s="24"/>
+      <c r="K3" s="24"/>
+    </row>
+    <row r="4" spans="1:11" s="5" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="B4" s="7"/>
+      <c r="C4" s="8"/>
+      <c r="D4" s="8"/>
+      <c r="E4" s="7"/>
+      <c r="F4" s="7"/>
+      <c r="G4" s="7"/>
+      <c r="H4" s="7"/>
+      <c r="I4" s="7"/>
+      <c r="J4" s="7"/>
+      <c r="K4" s="7"/>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A5" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="B4" s="7">
+      <c r="B5" s="7">
         <v>2</v>
       </c>
     </row>
-    <row r="5" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="20" t="s">
+    <row r="6" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A6" s="20" t="s">
+        <v>39</v>
+      </c>
+      <c r="B6" s="18" t="s">
+        <v>54</v>
+      </c>
+      <c r="C6" s="19"/>
+      <c r="D6" s="19"/>
+      <c r="E6" s="19"/>
+      <c r="F6" s="21" t="s">
+        <v>46</v>
+      </c>
+      <c r="G6" s="21" t="s">
+        <v>47</v>
+      </c>
+      <c r="H6" s="21" t="s">
+        <v>56</v>
+      </c>
+      <c r="I6" s="21" t="s">
+        <v>50</v>
+      </c>
+      <c r="J6" s="21" t="s">
+        <v>51</v>
+      </c>
+      <c r="K6" s="18" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" s="4" customFormat="1" ht="31.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A7" s="19"/>
+      <c r="B7" s="15" t="s">
+        <v>36</v>
+      </c>
+      <c r="C7" s="15" t="s">
+        <v>37</v>
+      </c>
+      <c r="D7" s="15" t="s">
+        <v>55</v>
+      </c>
+      <c r="E7" s="15" t="s">
+        <v>42</v>
+      </c>
+      <c r="F7" s="22"/>
+      <c r="G7" s="22"/>
+      <c r="H7" s="23"/>
+      <c r="I7" s="23"/>
+      <c r="J7" s="23"/>
+      <c r="K7" s="19"/>
+    </row>
+    <row r="8" spans="1:11" s="2" customFormat="1" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A8" s="16" t="s">
         <v>40</v>
       </c>
-      <c r="B5" s="18" t="s">
-        <v>55</v>
-      </c>
-      <c r="C5" s="19"/>
-      <c r="D5" s="19"/>
-      <c r="E5" s="19"/>
-      <c r="F5" s="21" t="s">
-        <v>47</v>
-      </c>
-      <c r="G5" s="21" t="s">
+      <c r="B8" s="10" t="s">
+        <v>35</v>
+      </c>
+      <c r="C8" s="10" t="s">
+        <v>38</v>
+      </c>
+      <c r="D8" s="10" t="s">
+        <v>41</v>
+      </c>
+      <c r="E8" s="11" t="s">
+        <v>43</v>
+      </c>
+      <c r="F8" s="11" t="s">
+        <v>49</v>
+      </c>
+      <c r="G8" s="11" t="s">
         <v>48</v>
       </c>
-      <c r="H5" s="21" t="s">
+      <c r="H8" s="11" t="s">
         <v>57</v>
       </c>
-      <c r="I5" s="21" t="s">
-        <v>51</v>
-      </c>
-      <c r="J5" s="21" t="s">
+      <c r="I8" s="17" t="s">
         <v>52</v>
       </c>
-      <c r="K5" s="18" t="s">
+      <c r="J8" s="17" t="s">
+        <v>53</v>
+      </c>
+      <c r="K8" s="12" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="6" spans="1:11" s="4" customFormat="1" ht="31.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="19"/>
-      <c r="B6" s="15" t="s">
-        <v>37</v>
-      </c>
-      <c r="C6" s="15" t="s">
-        <v>38</v>
-      </c>
-      <c r="D6" s="15" t="s">
-        <v>56</v>
-      </c>
-      <c r="E6" s="15" t="s">
-        <v>43</v>
-      </c>
-      <c r="F6" s="22"/>
-      <c r="G6" s="22"/>
-      <c r="H6" s="23"/>
-      <c r="I6" s="23"/>
-      <c r="J6" s="23"/>
-      <c r="K6" s="19"/>
-    </row>
-    <row r="7" spans="1:11" s="2" customFormat="1" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="16" t="s">
-        <v>41</v>
-      </c>
-      <c r="B7" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="C7" s="10" t="s">
-        <v>39</v>
-      </c>
-      <c r="D7" s="10" t="s">
-        <v>42</v>
-      </c>
-      <c r="E7" s="11" t="s">
-        <v>44</v>
-      </c>
-      <c r="F7" s="11" t="s">
-        <v>50</v>
-      </c>
-      <c r="G7" s="11" t="s">
-        <v>49</v>
-      </c>
-      <c r="H7" s="11" t="s">
-        <v>58</v>
-      </c>
-      <c r="I7" s="17" t="s">
-        <v>53</v>
-      </c>
-      <c r="J7" s="17" t="s">
-        <v>54</v>
-      </c>
-      <c r="K7" s="12" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="C9" s="13"/>
-      <c r="D9" s="13"/>
-      <c r="E9" s="14"/>
-      <c r="F9" s="14"/>
-      <c r="G9" s="14"/>
-      <c r="H9" s="14"/>
-      <c r="I9" s="14"/>
-      <c r="J9" s="14"/>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="C10" s="13"/>
+      <c r="D10" s="13"/>
+      <c r="E10" s="14"/>
+      <c r="F10" s="14"/>
+      <c r="G10" s="14"/>
+      <c r="H10" s="14"/>
+      <c r="I10" s="14"/>
+      <c r="J10" s="14"/>
     </row>
   </sheetData>
-  <mergeCells count="8">
-    <mergeCell ref="K5:K6"/>
-    <mergeCell ref="B5:E5"/>
-    <mergeCell ref="A5:A6"/>
-    <mergeCell ref="F5:F6"/>
-    <mergeCell ref="G5:G6"/>
-    <mergeCell ref="I5:I6"/>
-    <mergeCell ref="J5:J6"/>
-    <mergeCell ref="H5:H6"/>
+  <mergeCells count="9">
+    <mergeCell ref="A3:K3"/>
+    <mergeCell ref="K6:K7"/>
+    <mergeCell ref="B6:E6"/>
+    <mergeCell ref="A6:A7"/>
+    <mergeCell ref="F6:F7"/>
+    <mergeCell ref="G6:G7"/>
+    <mergeCell ref="I6:I7"/>
+    <mergeCell ref="J6:J7"/>
+    <mergeCell ref="H6:H7"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967292" verticalDpi="4294967292" r:id="rId1"/>

</xml_diff>

<commit_message>
fixing range filter by multiple assay
</commit_message>
<xml_diff>
--- a/api/templates/export/results/en.xlsx
+++ b/api/templates/export/results/en.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="24701"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="25225"/>
   <workbookPr showInkAnnotation="0" autoCompressPictures="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-20.04\home\ubuntu\aspect\api\templates\all_results\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\aepel\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{70F6B89A-9786-4A8E-A7AA-8CCDC0C77FF0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF4CA52E-AA33-49A9-9B06-CAD5D8B10D6B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5340" yWindow="5340" windowWidth="28800" windowHeight="15410" tabRatio="815" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-38020" yWindow="380" windowWidth="28800" windowHeight="15370" tabRatio="815" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Results" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="59">
   <si>
     <t>Code</t>
   </si>
@@ -136,12 +136,6 @@
     <t>&lt;stateName&gt;</t>
   </si>
   <si>
-    <t>State</t>
-  </si>
-  <si>
-    <t>LGA</t>
-  </si>
-  <si>
     <t>&lt;lgaName&gt;</t>
   </si>
   <si>
@@ -190,12 +184,6 @@
     <t>&lt;resultTreatmentStatus&gt;</t>
   </si>
   <si>
-    <t>Sample Collection Site</t>
-  </si>
-  <si>
-    <t>Site</t>
-  </si>
-  <si>
     <t>Error Code</t>
   </si>
   <si>
@@ -206,6 +194,15 @@
   </si>
   <si>
     <t>There are &lt;PerformanceTotalRecordLimit&gt; more records, but report size is limited to &lt;PerformanceQueryLimit&gt; records for performance reasons. If you need more results please filter them by any of the possible filters we are providing.</t>
+  </si>
+  <si>
+    <t>Sample State</t>
+  </si>
+  <si>
+    <t>Sample LGA</t>
+  </si>
+  <si>
+    <t>Sample Site</t>
   </si>
 </sst>
 </file>
@@ -287,7 +284,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="4">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -323,19 +320,6 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top/>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="44">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -383,7 +367,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -392,9 +376,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -437,23 +418,17 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="43" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="44">
@@ -865,183 +840,160 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K10"/>
+  <dimension ref="A1:K9"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="22.5" style="5" customWidth="1"/>
-    <col min="2" max="2" width="23.08203125" style="7" customWidth="1"/>
-    <col min="3" max="3" width="22.4140625" style="8" customWidth="1"/>
-    <col min="4" max="4" width="18.5" style="8" customWidth="1"/>
-    <col min="5" max="5" width="28.58203125" style="9" customWidth="1"/>
-    <col min="6" max="6" width="21.4140625" style="9" customWidth="1"/>
-    <col min="7" max="7" width="21.33203125" style="9" customWidth="1"/>
-    <col min="8" max="8" width="11.9140625" style="9" customWidth="1"/>
-    <col min="9" max="9" width="17.1640625" style="9" customWidth="1"/>
-    <col min="10" max="10" width="15.9140625" style="9" customWidth="1"/>
-    <col min="11" max="11" width="20.6640625" style="9" customWidth="1"/>
+    <col min="1" max="1" width="22.5" style="4" customWidth="1"/>
+    <col min="2" max="2" width="23.08203125" style="6" customWidth="1"/>
+    <col min="3" max="3" width="22.4140625" style="7" customWidth="1"/>
+    <col min="4" max="4" width="18.5" style="7" customWidth="1"/>
+    <col min="5" max="5" width="28.58203125" style="8" customWidth="1"/>
+    <col min="6" max="6" width="21.4140625" style="8" customWidth="1"/>
+    <col min="7" max="7" width="21.33203125" style="8" customWidth="1"/>
+    <col min="8" max="8" width="11.9140625" style="8" customWidth="1"/>
+    <col min="9" max="9" width="17.1640625" style="8" customWidth="1"/>
+    <col min="10" max="10" width="15.9140625" style="8" customWidth="1"/>
+    <col min="11" max="11" width="20.6640625" style="8" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="21" x14ac:dyDescent="0.5">
-      <c r="A1" s="6" t="s">
+      <c r="A1" s="5" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="2" spans="1:11" s="5" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="5" t="s">
+    <row r="2" spans="1:11" s="4" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="B2" s="6"/>
+      <c r="C2" s="7"/>
+      <c r="D2" s="7"/>
+      <c r="E2" s="6"/>
+      <c r="F2" s="6"/>
+      <c r="G2" s="6"/>
+      <c r="H2" s="6"/>
+      <c r="I2" s="6"/>
+      <c r="J2" s="6"/>
+      <c r="K2" s="6"/>
+    </row>
+    <row r="3" spans="1:11" s="4" customFormat="1" ht="29" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A3" s="18" t="s">
+        <v>55</v>
+      </c>
+      <c r="B3" s="18"/>
+      <c r="C3" s="18"/>
+      <c r="D3" s="18"/>
+      <c r="E3" s="18"/>
+      <c r="F3" s="18"/>
+      <c r="G3" s="18"/>
+      <c r="H3" s="18"/>
+      <c r="I3" s="18"/>
+      <c r="J3" s="18"/>
+      <c r="K3" s="18"/>
+    </row>
+    <row r="4" spans="1:11" s="4" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="B4" s="6"/>
+      <c r="C4" s="7"/>
+      <c r="D4" s="7"/>
+      <c r="E4" s="6"/>
+      <c r="F4" s="6"/>
+      <c r="G4" s="6"/>
+      <c r="H4" s="6"/>
+      <c r="I4" s="6"/>
+      <c r="J4" s="6"/>
+      <c r="K4" s="6"/>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A5" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="B5" s="6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A6" s="19" t="s">
+        <v>37</v>
+      </c>
+      <c r="B6" s="17" t="s">
+        <v>56</v>
+      </c>
+      <c r="C6" s="14" t="s">
+        <v>57</v>
+      </c>
+      <c r="D6" s="14" t="s">
         <v>58</v>
       </c>
-      <c r="B2" s="7"/>
-      <c r="C2" s="8"/>
-      <c r="D2" s="8"/>
-      <c r="E2" s="7"/>
-      <c r="F2" s="7"/>
-      <c r="G2" s="7"/>
-      <c r="H2" s="7"/>
-      <c r="I2" s="7"/>
-      <c r="J2" s="7"/>
-      <c r="K2" s="7"/>
-    </row>
-    <row r="3" spans="1:11" s="5" customFormat="1" ht="29" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="24" t="s">
-        <v>59</v>
-      </c>
-      <c r="B3" s="24"/>
-      <c r="C3" s="24"/>
-      <c r="D3" s="24"/>
-      <c r="E3" s="24"/>
-      <c r="F3" s="24"/>
-      <c r="G3" s="24"/>
-      <c r="H3" s="24"/>
-      <c r="I3" s="24"/>
-      <c r="J3" s="24"/>
-      <c r="K3" s="24"/>
-    </row>
-    <row r="4" spans="1:11" s="5" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="B4" s="7"/>
-      <c r="C4" s="8"/>
-      <c r="D4" s="8"/>
-      <c r="E4" s="7"/>
-      <c r="F4" s="7"/>
-      <c r="G4" s="7"/>
-      <c r="H4" s="7"/>
-      <c r="I4" s="7"/>
-      <c r="J4" s="7"/>
-      <c r="K4" s="7"/>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A5" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="B5" s="7">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="6" spans="1:11" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="20" t="s">
+      <c r="E6" s="14" t="s">
+        <v>40</v>
+      </c>
+      <c r="F6" s="21" t="s">
+        <v>44</v>
+      </c>
+      <c r="G6" s="21" t="s">
+        <v>45</v>
+      </c>
+      <c r="H6" s="21" t="s">
+        <v>52</v>
+      </c>
+      <c r="I6" s="21" t="s">
+        <v>48</v>
+      </c>
+      <c r="J6" s="21" t="s">
+        <v>49</v>
+      </c>
+      <c r="K6" s="20" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" s="2" customFormat="1" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A7" s="15" t="s">
+        <v>38</v>
+      </c>
+      <c r="B7" s="9" t="s">
+        <v>35</v>
+      </c>
+      <c r="C7" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="D7" s="9" t="s">
         <v>39</v>
       </c>
-      <c r="B6" s="18" t="s">
-        <v>54</v>
-      </c>
-      <c r="C6" s="19"/>
-      <c r="D6" s="19"/>
-      <c r="E6" s="19"/>
-      <c r="F6" s="21" t="s">
+      <c r="E7" s="10" t="s">
+        <v>41</v>
+      </c>
+      <c r="F7" s="10" t="s">
+        <v>47</v>
+      </c>
+      <c r="G7" s="10" t="s">
         <v>46</v>
       </c>
-      <c r="G6" s="21" t="s">
-        <v>47</v>
-      </c>
-      <c r="H6" s="21" t="s">
-        <v>56</v>
-      </c>
-      <c r="I6" s="21" t="s">
+      <c r="H7" s="10" t="s">
+        <v>53</v>
+      </c>
+      <c r="I7" s="16" t="s">
         <v>50</v>
       </c>
-      <c r="J6" s="21" t="s">
+      <c r="J7" s="16" t="s">
         <v>51</v>
       </c>
-      <c r="K6" s="18" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="7" spans="1:11" s="4" customFormat="1" ht="31.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="19"/>
-      <c r="B7" s="15" t="s">
-        <v>36</v>
-      </c>
-      <c r="C7" s="15" t="s">
-        <v>37</v>
-      </c>
-      <c r="D7" s="15" t="s">
-        <v>55</v>
-      </c>
-      <c r="E7" s="15" t="s">
-        <v>42</v>
-      </c>
-      <c r="F7" s="22"/>
-      <c r="G7" s="22"/>
-      <c r="H7" s="23"/>
-      <c r="I7" s="23"/>
-      <c r="J7" s="23"/>
-      <c r="K7" s="19"/>
-    </row>
-    <row r="8" spans="1:11" s="2" customFormat="1" ht="15.65" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="16" t="s">
-        <v>40</v>
-      </c>
-      <c r="B8" s="10" t="s">
-        <v>35</v>
-      </c>
-      <c r="C8" s="10" t="s">
-        <v>38</v>
-      </c>
-      <c r="D8" s="10" t="s">
-        <v>41</v>
-      </c>
-      <c r="E8" s="11" t="s">
+      <c r="K7" s="11" t="s">
         <v>43</v>
       </c>
-      <c r="F8" s="11" t="s">
-        <v>49</v>
-      </c>
-      <c r="G8" s="11" t="s">
-        <v>48</v>
-      </c>
-      <c r="H8" s="11" t="s">
-        <v>57</v>
-      </c>
-      <c r="I8" s="17" t="s">
-        <v>52</v>
-      </c>
-      <c r="J8" s="17" t="s">
-        <v>53</v>
-      </c>
-      <c r="K8" s="12" t="s">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="C10" s="13"/>
-      <c r="D10" s="13"/>
-      <c r="E10" s="14"/>
-      <c r="F10" s="14"/>
-      <c r="G10" s="14"/>
-      <c r="H10" s="14"/>
-      <c r="I10" s="14"/>
-      <c r="J10" s="14"/>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="C9" s="12"/>
+      <c r="D9" s="12"/>
+      <c r="E9" s="13"/>
+      <c r="F9" s="13"/>
+      <c r="G9" s="13"/>
+      <c r="H9" s="13"/>
+      <c r="I9" s="13"/>
+      <c r="J9" s="13"/>
     </row>
   </sheetData>
-  <mergeCells count="9">
+  <mergeCells count="1">
     <mergeCell ref="A3:K3"/>
-    <mergeCell ref="K6:K7"/>
-    <mergeCell ref="B6:E6"/>
-    <mergeCell ref="A6:A7"/>
-    <mergeCell ref="F6:F7"/>
-    <mergeCell ref="G6:G7"/>
-    <mergeCell ref="I6:I7"/>
-    <mergeCell ref="J6:J7"/>
-    <mergeCell ref="H6:H7"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967292" verticalDpi="4294967292" r:id="rId1"/>

</xml_diff>